<commit_message>
feat(forms): cascading selects + section-level skip logic (XLSForm import + renderer)
- Cascading selects: choices sheet may carry attribute columns and a survey
  `choice_filter` column (e.g. block=${block}); the parser stores them as
  option attrs + field.choiceFilter, and the renderer narrows a select's
  options by the parent field's answer. Village lists cascade Block->GP->Village.
- Section-level skip logic: `relevant` on a begin_group row now becomes the
  section's skipLogic, so a whole section can be hidden (e.g. hide all sections
  when consent = No). Renderer already honored shouldShowSection.
- Starter template updated with a state->district cascading example and the
  choice_filter column so users can author it and import via xlsx.

Needed for the Niiti Sangwari form (95 villages across 4 blocks + consent gate).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/FieldGovern_Form_Template.xlsx
+++ b/frontend/public/FieldGovern_Form_Template.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -437,6 +437,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,6 +486,11 @@
           <t>parameters</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>choice_filter</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -516,6 +522,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -543,6 +550,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -570,6 +578,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -597,6 +606,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -624,6 +634,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -651,6 +662,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -682,75 +694,86 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>geopoint</t>
+          <t>select_one state</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GPS location</t>
+          <t>State</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>select_one district</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>house_photo</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Photo of house</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Only districts in the chosen state show</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>state=${state}</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>barcode</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>hh_id</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Household barcode</t>
+          <t>GPS location</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -763,214 +786,279 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>thanks_note</t>
+          <t>house_photo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thank you for your time.</t>
+          <t>Photo of house</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>barcode</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>age_next_year</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>hh_id</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Household barcode</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>age + 1</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>range</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>satisfaction</t>
+          <t>thanks_note</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Satisfaction (1-5)</t>
+          <t>Thank you for your time.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>rating</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>start=1 end=5 step=1</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>num_children</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Number of children</t>
-        </is>
-      </c>
+          <t>age_next_year</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>age + 1</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>range</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>members</t>
+          <t>satisfaction</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Household members</t>
+          <t>Satisfaction (1-5)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>start=1 end=5 step=1</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>member_name</t>
+          <t>num_children</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Member name</t>
+          <t>Number of children</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>begin_repeat</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>member_age</t>
+          <t>members</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Member age</t>
+          <t>Household members</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>end_repeat</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>members</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>member_name</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Member name</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>member_age</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Member age</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>end_repeat</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>members</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -983,12 +1071,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1007,6 +1096,11 @@
           <t>label</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1024,6 +1118,7 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1041,6 +1136,7 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1058,6 +1154,7 @@
           <t>Other</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1075,6 +1172,7 @@
           <t>Fever / Malaria</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1092,6 +1190,7 @@
           <t>Cough / Respiratory</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1109,6 +1208,7 @@
           <t>Chronic (BP, diabetes)</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1124,6 +1224,131 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>None</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>mh</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>cg</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Chhattisgarh</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>pune</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>mh</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>nagpur</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Nagpur</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>mh</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>raipur</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>cg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>surguja</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Surguja</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>cg</t>
         </is>
       </c>
     </row>

</xml_diff>